<commit_message>
organizacao claude code 2
</commit_message>
<xml_diff>
--- a/PJA_RANKINGS_2026.xlsx
+++ b/PJA_RANKINGS_2026.xlsx
@@ -1369,10 +1369,10 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>213</v>
+        <v>192</v>
       </c>
       <c r="G6" s="2">
         <f>IF(J6="","",RANK(J6,$J$6:$J$14,0))</f>
@@ -1384,10 +1384,10 @@
         </is>
       </c>
       <c r="I6" s="2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>213</v>
+        <v>192</v>
       </c>
       <c r="L6" s="2">
         <f>IF(O6="","",RANK(O6,$O$6:$O$13,0))</f>
@@ -1399,10 +1399,10 @@
         </is>
       </c>
       <c r="N6" s="2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>163</v>
+        <v>149</v>
       </c>
     </row>
     <row r="7">
@@ -1416,10 +1416,10 @@
         </is>
       </c>
       <c r="D7" s="5" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>172</v>
+        <v>152</v>
       </c>
       <c r="G7" s="5">
         <f>IF(J7="","",RANK(J7,$J$6:$J$14,0))</f>
@@ -1427,14 +1427,14 @@
       </c>
       <c r="H7" s="6" t="inlineStr">
         <is>
-          <t>João Rocha</t>
+          <t>William Gao</t>
         </is>
       </c>
       <c r="I7" s="5" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>142</v>
+        <v>125</v>
       </c>
       <c r="L7" s="5">
         <f>IF(O7="","",RANK(O7,$O$6:$O$13,0))</f>
@@ -1442,14 +1442,14 @@
       </c>
       <c r="M7" s="6" t="inlineStr">
         <is>
-          <t>Angelina Gao</t>
+          <t>Rodrigo Correia</t>
         </is>
       </c>
       <c r="N7" s="5" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="O7" s="7" t="n">
-        <v>130</v>
+        <v>116</v>
       </c>
     </row>
     <row r="8">
@@ -1463,10 +1463,10 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>163</v>
+        <v>149</v>
       </c>
       <c r="G8" s="2">
         <f>IF(J8="","",RANK(J8,$J$6:$J$14,0))</f>
@@ -1474,14 +1474,14 @@
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>William Gao</t>
+          <t>João Rocha</t>
         </is>
       </c>
       <c r="I8" s="2" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>139</v>
+        <v>122</v>
       </c>
       <c r="L8" s="2">
         <f>IF(O8="","",RANK(O8,$O$6:$O$13,0))</f>
@@ -1489,14 +1489,14 @@
       </c>
       <c r="M8" s="3" t="inlineStr">
         <is>
-          <t>Rodrigo Correia</t>
+          <t>Angelina Gao</t>
         </is>
       </c>
       <c r="N8" s="2" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="O8" s="4" t="n">
-        <v>116</v>
+        <v>112</v>
       </c>
     </row>
     <row r="9">
@@ -1510,10 +1510,10 @@
         </is>
       </c>
       <c r="D9" s="5" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>139</v>
+        <v>125</v>
       </c>
       <c r="G9" s="5">
         <f>IF(J9="","",RANK(J9,$J$6:$J$14,0))</f>
@@ -1525,10 +1525,10 @@
         </is>
       </c>
       <c r="I9" s="5" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>134</v>
+        <v>116</v>
       </c>
       <c r="L9" s="5">
         <f>IF(O9="","",RANK(O9,$O$6:$O$13,0))</f>
@@ -1540,10 +1540,10 @@
         </is>
       </c>
       <c r="N9" s="5" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="O9" s="7" t="n">
-        <v>93</v>
+        <v>83</v>
       </c>
     </row>
     <row r="10">
@@ -1553,14 +1553,14 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Salvador Ivo de Carvalho</t>
+          <t>João Rocha</t>
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>134</v>
+        <v>122</v>
       </c>
       <c r="G10" s="2">
         <f>IF(J10="","",RANK(J10,$J$6:$J$14,0))</f>
@@ -1583,14 +1583,14 @@
       </c>
       <c r="M10" s="3" t="inlineStr">
         <is>
-          <t>Rafael Benesi</t>
+          <t>Diogo Sequeira</t>
         </is>
       </c>
       <c r="N10" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>63</v>
+        <v>49</v>
       </c>
     </row>
     <row r="11">
@@ -1600,14 +1600,14 @@
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Angelina Gao</t>
+          <t>Rodrigo Correia</t>
         </is>
       </c>
       <c r="D11" s="5" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>130</v>
+        <v>116</v>
       </c>
       <c r="G11" s="5">
         <f>IF(J11="","",RANK(J11,$J$6:$J$14,0))</f>
@@ -1619,10 +1619,10 @@
         </is>
       </c>
       <c r="I11" s="5" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>89</v>
+        <v>82</v>
       </c>
       <c r="L11" s="5">
         <f>IF(O11="","",RANK(O11,$O$6:$O$13,0))</f>
@@ -1630,14 +1630,14 @@
       </c>
       <c r="M11" s="6" t="inlineStr">
         <is>
-          <t>Diogo Sequeira</t>
+          <t>Rafael Benesi</t>
         </is>
       </c>
       <c r="N11" s="5" t="n">
         <v>4</v>
       </c>
       <c r="O11" s="7" t="n">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="12">
@@ -1647,11 +1647,11 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Rodrigo Correia</t>
+          <t>Salvador Ivo de Carvalho</t>
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E12" s="4" t="n">
         <v>116</v>
@@ -1677,14 +1677,14 @@
       </c>
       <c r="M12" s="3" t="inlineStr">
         <is>
-          <t>Clara Trindade</t>
+          <t>Ryan Dantas</t>
         </is>
       </c>
       <c r="N12" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O12" s="4" t="n">
-        <v>47</v>
+        <v>39</v>
       </c>
     </row>
     <row r="13">
@@ -1694,14 +1694,14 @@
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>Santiago Dias</t>
+          <t>Angelina Gao</t>
         </is>
       </c>
       <c r="D13" s="5" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="G13" s="5">
         <f>IF(J13="","",RANK(J13,$J$6:$J$14,0))</f>
@@ -1724,14 +1724,14 @@
       </c>
       <c r="M13" s="6" t="inlineStr">
         <is>
-          <t>Ryan Dantas</t>
+          <t>Clara Trindade</t>
         </is>
       </c>
       <c r="N13" s="5" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="O13" s="7" t="n">
-        <v>39</v>
+        <v>32</v>
       </c>
     </row>
     <row r="14">
@@ -1741,14 +1741,14 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Rodrigo Constantino</t>
+          <t>Santiago Dias</t>
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="G14" s="5">
         <f>IF(J14="","",RANK(J14,$J$6:$J$14,0))</f>
@@ -1773,14 +1773,14 @@
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>Madalena Figueiredo</t>
+          <t>Rodrigo Constantino</t>
         </is>
       </c>
       <c r="D15" s="5" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>93</v>
+        <v>105</v>
       </c>
       <c r="G15" s="11" t="inlineStr">
         <is>
@@ -1857,14 +1857,14 @@
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>David Filip</t>
+          <t>João Maria Ivo de Carvalho</t>
         </is>
       </c>
       <c r="D17" s="5" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="G17" s="2">
         <f>IF(J17="","",RANK(J17,$J$17:$J$20,0))</f>
@@ -1876,10 +1876,10 @@
         </is>
       </c>
       <c r="I17" s="2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J17" s="4" t="n">
-        <v>172</v>
+        <v>152</v>
       </c>
       <c r="L17" s="2">
         <f>IF(O17="","",RANK(O17,$O$17:$O$18,0))</f>
@@ -1904,11 +1904,11 @@
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>João Maria Ivo de Carvalho</t>
+          <t>Madalena Figueiredo</t>
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="E18" s="4" t="n">
         <v>83</v>
@@ -1951,14 +1951,14 @@
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>Ziyang Guo</t>
+          <t>David Filip</t>
         </is>
       </c>
       <c r="D19" s="5" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E19" s="7" t="n">
-        <v>71</v>
+        <v>82</v>
       </c>
       <c r="G19" s="2">
         <f>IF(J19="","",RANK(J19,$J$17:$J$20,0))</f>
@@ -1983,14 +1983,14 @@
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>Rafael Benesi</t>
+          <t>Ziyang Guo</t>
         </is>
       </c>
       <c r="D20" s="2" t="n">
         <v>5</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>63</v>
+        <v>71</v>
       </c>
       <c r="G20" s="5">
         <f>IF(J20="","",RANK(J20,$J$17:$J$20,0))</f>
@@ -2057,7 +2057,7 @@
         </is>
       </c>
       <c r="D23" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E23" s="7" t="n">
         <v>49</v>
@@ -2070,11 +2070,11 @@
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>Clara Trindade</t>
+          <t>Rafael Benesi</t>
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E24" s="4" t="n">
         <v>47</v>
@@ -2121,14 +2121,14 @@
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>Francisco Carvalho</t>
+          <t>Clara Trindade</t>
         </is>
       </c>
       <c r="D27" s="5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E27" s="7" t="n">
-        <v>14</v>
+        <v>32</v>
       </c>
     </row>
     <row r="28">
@@ -2138,14 +2138,14 @@
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>Martim Shipitsyn Moreira</t>
+          <t>Francisco Carvalho</t>
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E28" s="4" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="29">
@@ -2155,11 +2155,11 @@
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>Rafaela Pinto</t>
+          <t>Martim Shipitsyn Moreira</t>
         </is>
       </c>
       <c r="D29" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E29" s="7" t="n">
         <v>11</v>
@@ -2172,11 +2172,15 @@
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>Emile Cuanalo</t>
-        </is>
-      </c>
-      <c r="D30" s="2" t="n"/>
-      <c r="E30" s="4" t="n"/>
+          <t>Rafaela Pinto</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E30" s="4" t="n">
+        <v>11</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="7">

</xml_diff>